<commit_message>
update page creation excel
</commit_message>
<xml_diff>
--- a/templates/seiten-erstellen_b.xlsx
+++ b/templates/seiten-erstellen_b.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.roe.AD\Documents\Code\online-exerzitien\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48C4956A-085F-4784-8CF4-DB27B870C913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21572EED-CDC4-4DB5-AA7F-DBC3D05BE7A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1C311BB0-7E16-43E4-97F4-7A8195C78B44}"/>
   </bookViews>
@@ -21526,7 +21526,7 @@
         <v>71</v>
       </c>
       <c r="D27" s="6" t="str">
-        <f>header_block_de!A1</f>
+        <f>header_block_de!$A1</f>
         <v>&lt;header class="site-header"&gt;
       &lt;div class="cover-img"&gt;
                 &lt;img src="/img/website_banner.jpg" alt="Heiligen des Karmels"&gt;
@@ -21635,9 +21635,115 @@
 &lt;/div&gt;
       &lt;/nav&gt;</v>
       </c>
-      <c r="E27" s="8">
-        <f>header_block_de!B1</f>
-        <v>0</v>
+      <c r="E27" s="6" t="str">
+        <f>header_block_de!$A1</f>
+        <v>&lt;header class="site-header"&gt;
+      &lt;div class="cover-img"&gt;
+                &lt;img src="/img/website_banner.jpg" alt="Heiligen des Karmels"&gt;
+&lt;/div&gt;
+      &lt;/div&gt;
+    &lt;/header&gt;
+      &lt;nav class="header-inner"&gt;
+        &lt;a href="#" class="brand" aria-label="Startseite"&gt;
+          &lt;span class="brand-mark" aria-hidden="true"&gt;&lt;img src="/img/apple-touch-icon.png" style="border-radius: var(--radius-lg)"&gt;&lt;/span&gt;
+          &lt;span class="brand-text"&gt;
+            &lt;span class="brand-kicker"&gt;Karmel&lt;/span&gt;
+            &lt;span class="brand-name"&gt;Online-Exerzitien&lt;/span&gt;
+          &lt;/span&gt;
+        &lt;/a&gt;
+&lt;div class="header-actions"&gt;
+  &lt;details class="language-menu"&gt;
+    &lt;summary class="language-menu__trigger" aria-label="Sprache auswählen"&gt;
+      &lt;span aria-hidden="true"&gt;🌐&lt;/span&gt;
+      &lt;span&gt;DE&lt;/span&gt;
+      &lt;span class="language-menu__current"&gt;Deutsch&lt;/span&gt;
+    &lt;/summary&gt;
+    &lt;nav class="language-menu__list" aria-label="Sprachauswahl"&gt;
+      &lt;a href="https://retraites.carmes-paris.org/" lang="fr" hreflang="fr"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇫🇷&lt;/span&gt;
+        &lt;span class="language-code"&gt;FR&lt;/span&gt;
+        &lt;span&gt;Français&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/de/" lang="de" hreflang="de" aria-current="page"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇦🇹🇩🇪&lt;/span&gt;
+        &lt;span class="language-code"&gt;DE&lt;/span&gt;
+        &lt;span&gt;Deutsch&lt;/span&gt;
+        &lt;span class="language-check" aria-hidden="true"&gt;✓&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/es/" lang="es" hreflang="es"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇪🇸&lt;/span&gt;
+        &lt;span class="language-code"&gt;ES&lt;/span&gt;
+        &lt;span&gt;Español&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/it/" lang="it" hreflang="it"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇮🇹&lt;/span&gt;
+        &lt;span class="language-code"&gt;IT&lt;/span&gt;
+        &lt;span&gt;Italiano&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/en/" lang="en" hreflang="en"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇬🇧🇺🇸&lt;/span&gt;
+        &lt;span class="language-code"&gt;EN&lt;/span&gt;
+        &lt;span&gt;English&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/pl/" lang="pl" hreflang="pl"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇵🇱&lt;/span&gt;
+        &lt;span class="language-code"&gt;PL&lt;/span&gt;
+        &lt;span&gt;Polski&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/ar/" lang="ar" hreflang="ar" dir="rtl"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇱🇧🇸🇦&lt;/span&gt;
+        &lt;span class="language-code"&gt;AR&lt;/span&gt;
+        &lt;span&gt;العربية&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/pt/" lang="pt" hreflang="pt"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇵🇹&lt;/span&gt;
+        &lt;span class="language-code"&gt;PT&lt;/span&gt;
+        &lt;span&gt;Português&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/zh/" lang="zh" hreflang="zh"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇨🇳&lt;/span&gt;
+        &lt;span class="language-code"&gt;ZH&lt;/span&gt;
+        &lt;span&gt;中文&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/cs/" lang="cs" hreflang="cs"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇨🇿&lt;/span&gt;
+        &lt;span class="language-code"&gt;CS&lt;/span&gt;
+        &lt;span&gt;Čeština&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/hr/" lang="hr" hreflang="hr"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇭🇷&lt;/span&gt;
+        &lt;span class="language-code"&gt;HR&lt;/span&gt;
+        &lt;span&gt;Hrvatski&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/hu/" lang="hu" hreflang="hu"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇭🇺&lt;/span&gt;
+        &lt;span class="language-code"&gt;HU&lt;/span&gt;
+        &lt;span&gt;Magyar&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/mt/" lang="mt" hreflang="mt"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇲🇹&lt;/span&gt;
+        &lt;span class="language-code"&gt;MT&lt;/span&gt;
+        &lt;span&gt;Malti&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/nl/" lang="nl" hreflang="nl"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇳🇱&lt;/span&gt;
+        &lt;span class="language-code"&gt;NL&lt;/span&gt;
+        &lt;span&gt;Nederlands&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/ro/" lang="ro" hreflang="ro"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇷🇴&lt;/span&gt;
+        &lt;span class="language-code"&gt;RO&lt;/span&gt;
+        &lt;span&gt;Română&lt;/span&gt;
+      &lt;/a&gt;
+      &lt;a href="/vi/" lang="vi" hreflang="vi"&gt;
+        &lt;span class="language-flag" aria-hidden="true"&gt;🇻🇳&lt;/span&gt;
+        &lt;span class="language-code"&gt;VI&lt;/span&gt;
+        &lt;span&gt;Tiếng Việt&lt;/span&gt;
+      &lt;/a&gt;
+    &lt;/nav&gt;
+  &lt;/details&gt;
+&lt;/div&gt;
+      &lt;/nav&gt;</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>71</v>
@@ -25548,7 +25654,7 @@
         <v>208</v>
       </c>
       <c r="D113" s="6" t="str">
-        <f>form_block_de!A1</f>
+        <f>form_block_de!$A1</f>
         <v>&lt;section class="section-intro" id="abonniere"&gt;
 &lt;div id="mc_embed_shell"&gt;  
 &lt;div id="mc_embed_signup"&gt;
@@ -25632,9 +25738,90 @@
         &lt;/div&gt;
       &lt;/section&gt;</v>
       </c>
-      <c r="E113" s="8">
-        <f>form_block_de!B1</f>
-        <v>0</v>
+      <c r="E113" s="6" t="str">
+        <f>form_block_de!$A1</f>
+        <v>&lt;section class="section-intro" id="abonniere"&gt;
+&lt;div id="mc_embed_shell"&gt;  
+&lt;div id="mc_embed_signup"&gt;
+    &lt;form action="https://karmel.us6.list-manage.com/subscribe/post?u=7c9d2aa0ecc1fde64fd44bc67&amp;amp;id=10430a5833&amp;amp;f_id=009254e3f0" method="post" id="mc-embedded-subscribe-form" name="mc-embedded-subscribe-form" class="validate" target="_self" novalidate=""&gt;
+        &lt;div id="mc_embed_signup_scroll"&gt;
+            &lt;div class="mc-field-group"&gt;&lt;label for="mce-EMAIL"&gt;eMail Adresse&lt;span class="asterisk"&gt;* (erforderlich)&lt;/span&gt;&lt;/label&gt;
+              &lt;input type="email" name="EMAIL" class="required email" id="mce-EMAIL" required="" value=""&gt;&lt;/div&gt;
+              &lt;div class="mc-field-group"&gt;&lt;label for="mce-FNAME"&gt;Vorname &lt;/label&gt;
+                &lt;input type="text" name="FNAME" class=" text" id="mce-FNAME" value=""&gt;&lt;/div&gt;
+                &lt;div class="mc-field-group"&gt;&lt;label for="mce-LNAME"&gt;Nachname &lt;/label&gt;
+                  &lt;input type="text" name="LNAME" class=" text" id="mce-LNAME" value=""&gt;&lt;/div&gt;
+                                        &lt;div class="mc-field-group"&gt;&lt;label for="mce-AUFMERKS01"&gt;Wie sind Sie auf uns aufmerksam geworden? &lt;/label&gt;
+                        &lt;select name="AUFMERKS01" class="" id="mce-AUFMERKS01"&gt;
+                        &lt;option value="Bitte auswahlen..."&gt;Bitte auswahlen...&lt;/option&gt;
+                        &lt;option value="Karmeliten in Wien"&gt;Karmeliten in Wien&lt;/option&gt;
+                        &lt;option value="Karmeliten in Linz"&gt;Karmeliten in Linz&lt;/option&gt;
+                        &lt;option value="Karmeliten in Graz"&gt;Karmeliten in Graz&lt;/option&gt;
+                        &lt;option value="Persönliche Empfehlung"&gt;Persönliche Empfehlung&lt;/option&gt;
+                        &lt;option value="Plakat"&gt;Plakat&lt;/option&gt;
+                        &lt;option value="Internetsuche"&gt;Internetsuche&lt;/option&gt;
+                        &lt;option value="YouTube"&gt;YouTube&lt;/option&gt;
+                        &lt;option value="Facebook"&gt;Facebook&lt;/option&gt;
+                        &lt;option value="Instagram"&gt;Instagram&lt;/option&gt;
+                        &lt;option value="Sonstiges"&gt;Sonstiges&lt;/option&gt;&lt;/select&gt;&lt;/div&gt;
+                      &lt;div class="mc-field-group" id="sonstiges-field" style="display:none"&gt;&lt;label for="mce-AUFMERKS02"&gt;Sonstiges&lt;/label&gt;
+                        &lt;input type="text" name="AUFMERKS02" class=" text" id="mce-AUFMERKS02" value="" disabled&gt;&lt;span id="mce-AUFMERKS02-HELPERTEXT" class="help-block" hidden&gt;Wenn Sie „Sonstiges“ ausgewählt haben, geben Sie bitte hier &lt;/span&gt;
+                      &lt;/div&gt;
+                  &lt;div class="mc-field-group"&gt;&lt;label for="mce-LNAME"&gt; &lt;/label&gt;
+                  &lt;/div&gt;
+                    &lt;div class="mc-field-group input-group"&gt;
+                      &lt;details class="interest-details"&gt;
+                        &lt;summary&gt;Weitere Angebote der Karmeliten&lt;/summary&gt;
+                        &lt;ul class="interest-group" style="text-align: left;"&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][64]" id="mce-group[16777]-16777-0" value=""&gt;&lt;label for="mce-group[16777]-16777-0"&gt;alle Veranstaltungen des Karmel in Österreich&lt;/label&gt;&lt;/li&gt;
+                          &lt;details class="interest-details" style="padding-left: 1rem"&gt;&lt;summary&gt;Orte und Formate einschränken&lt;/summary&gt;
+                            &lt;ul&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][512]" id="mce-group[16777]-16777-1" value="" &gt;&lt;label for="mce-group[16777]-16777-1"&gt;in Wien&lt;/label&gt;&lt;/li&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][1024]" id="mce-group[16777]-16777-2" value="" &gt;&lt;label for="mce-group[16777]-16777-2"&gt;in Linz&lt;/label&gt;&lt;/li&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][2048]" id="mce-group[16777]-16777-3" value="" &gt;&lt;label for="mce-group[16777]-16777-3"&gt;in Graz&lt;/label&gt;&lt;/li&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][524288]" id="mce-group[16777]-16777-4" value=""&gt;&lt;label for="mce-group[16777]-16777-4"&gt;online&lt;/label&gt;&lt;/li&gt;
+                      &lt;/ul&gt;
+                      &lt;/details&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][256]" id="mce-group[16777]-16777-5" value=""&gt;&lt;label for="mce-group[16777]-16777-5"&gt;Infos/Veranstaltungen der Edith Stein Gesellschaft&lt;/label&gt;&lt;/li&gt;
+                        &lt;details class="interest-details" &gt;&lt;summary&gt;Novenen und Exerzitien auswählen&lt;/summary&gt;
+                          &lt;ul&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][128]" id="mce-group[16777]-16777-6" value=""&gt;&lt;label for="mce-group[16777]-16777-6"&gt;Friedensgebet/Novene Hl. Edith Stein&lt;/label&gt;&lt;/li&gt;
+                        &lt;li style="display:none"&gt;&lt;input type="checkbox" name="group[16777][32]" id="mce-group[16777]-16777-7" value="" checked&gt;&lt;label for="mce-group[16777]-16777-7"&gt;Exerzitien Online in Advent/Fastenzeit&lt;/label&gt;&lt;/li&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][16]" id="mce-group[16777]-16777-8" value=""&gt;&lt;label for="mce-group[16777]-16777-8"&gt;Novene Online zum Skapulierfest&lt;/label&gt;&lt;/li&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][8192]" id="mce-group[16777]-16777-9" value=""&gt;&lt;label for="mce-group[16777]-16777-9"&gt;33 Schritte mit Maria zu Jesus&lt;/label&gt;&lt;/li&gt;
+                        &lt;li&gt;&lt;input type="checkbox" name="group[16777][4096]" id="mce-group[16777]-16777-10" value=""&gt;&lt;label for="mce-group[16777]-16777-10"&gt;Jesus-Gebet&lt;/label&gt;&lt;/li&gt;                      
+                          &lt;/ul&gt;
+                        &lt;/details&gt;
+&lt;!--                                    &lt;div class="card-links"&gt;
+              &lt;a href="#angebote-cards"&gt;Mehr Informationen zur Angebote nach unten&lt;/a&gt;
+            &lt;/div&gt; --&gt;
+                      &lt;/ul&gt;
+                      &lt;/details&gt;
+                      &lt;div hidden=""&gt;&lt;input type="hidden" name="tags" value="8501"&gt;&lt;/div&gt;
+                    &lt;/div&gt;
+        &lt;div id="mce-responses" class="clear"&gt;
+            &lt;div class="response" id="mce-error-response" style="display: none;"&gt;&lt;/div&gt;
+            &lt;div class="response" id="mce-success-response" style="display: none;"&gt;&lt;/div&gt;
+        &lt;/div&gt;&lt;div style="position: absolute; left: -5000px;" aria-hidden="true"&gt;&lt;input type="text" name="b_7c9d2aa0ecc1fde64fd44bc67_10430a5833" tabindex="-1" value=""&gt;&lt;/div&gt;
+        &lt;div class="clear"&gt;&lt;input type="submit" name="subscribe" id="mc-embedded-subscribe" class="button-signup" value="Anmelden"&gt;&lt;/div&gt;
+&lt;/form&gt;
+      &lt;/section&gt;
+                &lt;/div&gt;
+            &lt;/div&gt;
+                      &lt;div class="datenschutz-toggle"&gt;
+          &lt;a href="#datenschutz-wrap" id="datenschutz-toggle" aria-expanded="false" aria-controls="datenschutz-wrap"&gt;Datenschutz&lt;/a&gt;
+                      &lt;div id="datenschutz-wrap" hidden&gt;
+          &lt;p style="font-size: 14px;"&gt;Die Karmeliten in Österreich werden die Informationen, die Sie in diesem Formular angeben, dazu verwenden, mit Ihnen in Kontakt zu bleiben und Ihnen Informationen über Internet-Aktivitäten wie Exerzitien Online o.ä. zu übermitteln – je nach Ihrer Auswahl im obigen Formular.
+            Sie können Ihre Meinung jederzeit ändern, indem Sie auf den Abbestellungs-Link klicken, den Sie in der Fußzeile jeder E-Mail, die Sie von uns erhalten, finden können, oder indem Sie uns unter online-exerzitien@karmel.at kontaktieren. Wir werden Ihre Informationen mit Sorgfalt und Respekt behandeln. Weitere Informationen zu unseren Datenschutzpraktiken finden Sie auf unserer Website www.karmel.at. Indem Sie unten klicken, erklären Sie sich damit einverstanden, dass wir Ihre Informationen in Übereinstimmung mit diesen Bedingungen verarbeiten dürfen.
+          &lt;/p&gt;
+          &lt;p style="font-size: 14px;"&gt;
+  Wir nutzen Mailchimp als unsere Marketing-Plattform. Mit einem Klick auf den untenstehenden Button zum Abonnieren erklären Sie sich damit einverstanden, dass Ihre Daten zur Verarbeitung an Mailchimp übermittelt werden.&lt;/p&gt;
+  &lt;a class="plain-link" href="https://mailchimp.com/legal/terms/" target="_blank" rel="noopener noreferrer" style="display:inline-block; font-size: 14px; font-weight: 200; text-decoration:none;"&gt;
+      Mehr über die Datenschutzpraktiken von Mailchimp erfahren Sie hier.
+  &lt;/a&gt;&lt;/div&gt;&lt;/div&gt;
+          &lt;/div&gt;
+        &lt;/div&gt;
+      &lt;/section&gt;</v>
       </c>
       <c r="F113" s="6" t="s">
         <v>178</v>

</xml_diff>

<commit_message>
adding de 2022_ad and 2023_fs
</commit_message>
<xml_diff>
--- a/templates/seiten-erstellen_b.xlsx
+++ b/templates/seiten-erstellen_b.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.roe.AD\Documents\Code\online-exerzitien\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C9CFF1-A87E-4848-A6D4-50D0C49C1EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931E244B-79D1-4397-A09F-02EABFD60648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exerzitien_archive_de" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5918" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5922" uniqueCount="643">
   <si>
     <t>2024_ad</t>
   </si>
@@ -22809,6 +22809,21 @@
   </si>
   <si>
     <t>2023_lent</t>
+  </si>
+  <si>
+    <t>2023-01-01</t>
+  </si>
+  <si>
+    <t>2022-11-23</t>
+  </si>
+  <si>
+    <t>2022-03-02</t>
+  </si>
+  <si>
+    <t>2022-04-24</t>
+  </si>
+  <si>
+    <t>&lt;section class="section"&gt;</t>
   </si>
 </sst>
 </file>
@@ -22930,7 +22945,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -22955,6 +22970,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -23901,13 +23917,13 @@
         <f t="array" ref="G8">INDEX('exerzitien-katalog'!$F:$F,COLUMN(G8)+1)</f>
         <v>2023-02-22</v>
       </c>
-      <c r="H8">
+      <c r="H8" t="str">
         <f t="array" ref="H8">INDEX('exerzitien-katalog'!$F:$F,COLUMN(H8)+1)</f>
-        <v>0</v>
-      </c>
-      <c r="I8">
+        <v>2022-11-23</v>
+      </c>
+      <c r="I8" t="str">
         <f t="array" ref="I8">INDEX('exerzitien-katalog'!$F:$F,COLUMN(I8)+1)</f>
-        <v>0</v>
+        <v>2022-03-02</v>
       </c>
       <c r="J8" t="str">
         <f t="array" ref="J8">INDEX('exerzitien-katalog'!$F:$F,COLUMN(J8)+1)</f>
@@ -24019,13 +24035,13 @@
         <f t="array" ref="G9">INDEX('exerzitien-katalog'!$G:$G,COLUMN(G9)+1)</f>
         <v>2023-04-16</v>
       </c>
-      <c r="H9">
+      <c r="H9" t="str">
         <f t="array" ref="H9">INDEX('exerzitien-katalog'!$G:$G,COLUMN(H9)+1)</f>
-        <v>0</v>
-      </c>
-      <c r="I9">
+        <v>2023-01-01</v>
+      </c>
+      <c r="I9" t="str">
         <f t="array" ref="I9">INDEX('exerzitien-katalog'!$G:$G,COLUMN(I9)+1)</f>
-        <v>0</v>
+        <v>2022-04-24</v>
       </c>
       <c r="J9" t="str">
         <f t="array" ref="J9">INDEX('exerzitien-katalog'!$G:$G,COLUMN(J9)+1)</f>
@@ -29563,94 +29579,94 @@
     </row>
     <row r="58" spans="2:31" x14ac:dyDescent="0.25">
       <c r="B58" s="4" t="s">
-        <v>92</v>
+        <v>642</v>
       </c>
       <c r="C58" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="D58" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="O58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="P58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="Q58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="R58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="S58" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="T58" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="U58" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="V58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="W58" s="2" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="X58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="Y58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="Z58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="AA58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="AB58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="AC58" s="1" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="AD58" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
       <c r="AE58" t="s">
-        <v>93</v>
+        <v>642</v>
       </c>
     </row>
     <row r="59" spans="2:31" x14ac:dyDescent="0.25">
@@ -30036,11 +30052,11 @@
       </c>
       <c r="H63" s="1" t="str">
         <f t="shared" si="12"/>
-        <v>&lt;h3&gt;Vom 0. Jänner 1900 bis 0. Jänner 1900&lt;/h3&gt;</v>
+        <v>&lt;h3&gt;Vom 23. November 2022 bis 1. Jänner 2023&lt;/h3&gt;</v>
       </c>
       <c r="I63" s="1" t="str">
         <f t="shared" si="12"/>
-        <v>&lt;h3&gt;Vom 0. Jänner 1900 bis 0. Jänner 1900&lt;/h3&gt;</v>
+        <v>&lt;h3&gt;Vom 2. März 2022 bis 24. April 2022&lt;/h3&gt;</v>
       </c>
       <c r="J63" s="1" t="str">
         <f t="shared" ref="J63:U63" si="13">"&lt;h3&gt;Vom "&amp;TEXT(J8,"t. MMMM JJJJ")&amp;" bis "&amp;TEXT(J9,"t. MMMM JJJJ")&amp;"&lt;/h3&gt;"</f>
@@ -41088,7 +41104,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -41471,6 +41487,12 @@
       <c r="E9" t="s">
         <v>468</v>
       </c>
+      <c r="F9" s="10" t="s">
+        <v>639</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>638</v>
+      </c>
       <c r="H9" t="s">
         <v>478</v>
       </c>
@@ -41502,6 +41524,12 @@
       </c>
       <c r="E10" t="s">
         <v>468</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>641</v>
       </c>
       <c r="H10" t="s">
         <v>485</v>
@@ -42571,9 +42599,9 @@
         <f>'exerzitien-katalog'!$F8</f>
         <v>2023-02-22</v>
       </c>
-      <c r="H8">
+      <c r="H8" t="str">
         <f>'exerzitien-katalog'!$F9</f>
-        <v>0</v>
+        <v>2022-11-23</v>
       </c>
       <c r="I8" t="str">
         <f>'exerzitien-katalog'!$F7</f>
@@ -42637,9 +42665,9 @@
         <f>'exerzitien-katalog'!$G8</f>
         <v>2023-04-16</v>
       </c>
-      <c r="H9">
+      <c r="H9" t="str">
         <f>'exerzitien-katalog'!$G9</f>
-        <v>0</v>
+        <v>2023-01-01</v>
       </c>
       <c r="I9" t="str">
         <f>'exerzitien-katalog'!$G7</f>
@@ -45380,7 +45408,7 @@
       </c>
       <c r="H63" s="1" t="str">
         <f t="shared" si="3"/>
-        <v>&lt;h3&gt;Vom 0. Jänner bis 0. Jänner 1900&lt;/h3&gt;</v>
+        <v>&lt;h3&gt;Vom 23. November bis 1. Jänner 2023&lt;/h3&gt;</v>
       </c>
       <c r="I63" s="1" t="str">
         <f t="shared" si="3"/>

</xml_diff>